<commit_message>
feat(excel): autogeneracion inteligente de codigo y nombre de carro segun estandares Goodyear
</commit_message>
<xml_diff>
--- a/plantilla_carros_goodyear.xlsx
+++ b/plantilla_carros_goodyear.xlsx
@@ -449,192 +449,237 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>codigo_carro</t>
+          <t>tipo_carro</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>nombre_carro</t>
+          <t>turno_o_numero</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>categoria</t>
+          <t>area</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>supervisor</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>supervisor</t>
+          <t>ubicacion_especifica</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ubicacion_especifica</t>
+          <t>gaveta_1_herramientas</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>gaveta_1_herramientas</t>
+          <t>gaveta_2_herramientas</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>gaveta_2_herramientas</t>
+          <t>gaveta_3_herramientas</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>gaveta_3_herramientas</t>
+          <t>gaveta_4_herramientas</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>gaveta_4_herramientas</t>
+          <t>gaveta_5_herramientas</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>gaveta_5_herramientas</t>
+          <t>codigo_carro_opcional</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CH-ASRS-TA</t>
+          <t>TURNO</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Carro Turno A (ASRS)</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>TURNO</t>
+          <t>ASRS</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Área ASRS</t>
+          <t>Juanito Arias</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Juanito Arias</t>
+          <t>Pasillo Principal Bahía 1</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Pasillo Principal Bahía 1</t>
+          <t>Juego Llaves Combinadas 8-24mm, Chicharra 1/2", Dados de Impacto 17-21mm</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Juego Llaves Combinadas 8-24mm, Chicharra 1/2", Dados de Impacto 17-21mm</t>
+          <t>Destornillador Paleta 6x100mm, Destornillador Cruz PH2, Alicate Universal 8"</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Destornillador Paleta 6x100mm, Destornillador Cruz PH2, Alicate Universal 8"</t>
+          <t>Martillo de Bola 500g, Martillo de Goma, Cincel Plano, Cepillo de Acero</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Martillo de Bola 500g, Martillo de Goma, Cincel Plano, Cepillo de Acero</t>
+          <t>Cinta Métrica 5m, Flexómetro de Trabajo, Manguera Neumática, Pistola de Aire</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Cinta Métrica 5m, Flexómetro de Trabajo, Manguera Neumática, Pistola de Aire</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
           <t>Candados LOTO Rojos (2 un), Pinza Bloqueo, Tarjeta 5S, Gafas de Seguridad</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CH-CST-M01</t>
+          <t>MECANICO</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Carro Mecánico 01 (Construcción)</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>MECANICO</t>
+          <t>Construcción</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Área Construcción</t>
+          <t>Juanito Arias</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Bahía Mantenimiento Construcción</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Juego Dados 1/2" Heavy Duty (8-32mm), Chicharra Pesada 1/2", Palanca de Fuerza</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Extractor de Rodamientos 3 Patas, Llaves Corona 10-24mm, Llave Ajustable 12"</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Arco de Sierra Profesional, Cinceles Planos, Limas de Ajuste, Llave Stilson 14"</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Pistola Neumática de Impacto 1/2", Manómetro Digital, Aceite Lubricante</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Torquímetro Calibrado 1/2" (20-200 Nm), Pie de Metro Digital, Kit LOTO</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ELECTRICO</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Final Finish</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>Juanito Arias</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Bahía Mantenimiento Construcción</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Juego Dados 1/2" Heavy Duty (8-32mm), Chicharra Pesada 1/2", Palanca de Fuerza</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Extractor de Rodamientos 3 Patas, Llaves Corona 10-24mm, Llave Ajustable 12"</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Arco de Sierra Profesional, Cinceles Planos, Limas de Ajuste, Llave Stilson 14"</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Pistola Neumática de Impacto 1/2", Manómetro Digital, Aceite Lubricante</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Torquímetro Calibrado 1/2" (20-200 Nm), Pie de Metro Digital, Kit LOTO</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Bahía Eléctrica Final Finish</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Juego Destornilladores 1000V VDE (PH0-PH3, SL3-SL6), Pelacables Automático</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Multímetro Digital Fluke Calibrado, Pinza Amperimétrica True RMS</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Crimpador Terminales Eléctricos, Alicate de Punta VDE, Cautín 60W</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Guantes Dieléctricos Clase 0 (1000V), Detector de Tensión Sin Contacto</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Candados LOTO Dieléctricos, Tarjetas de Advertencia Eléctrica, Lentes</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>